<commit_message>
Clean sample data and update project files
</commit_message>
<xml_diff>
--- a/JobTracker.xlsx
+++ b/JobTracker.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Github\Job Tracker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url=""/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{0C388516-5DA9-47C3-A5AC-99ADEC811556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -48,21 +48,21 @@
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
   <connection id="1" xr16:uid="{2D273CAE-9C45-49C4-A26E-BB161CF0738C}" interval="1" name="applications" type="6" refreshedVersion="8" refreshOnLoad="1" saveData="1">
-    <textPr prompt="0" sourceFile="C:\Users\user\Desktop\Github\Job Tracker\applications.csv" comma="1">
+    <textPr prompt="0" sourceFile="applications.csv" comma="1">
       <textFields>
         <textField/>
       </textFields>
     </textPr>
   </connection>
   <connection id="2" xr16:uid="{E15A7276-8443-4255-93A1-EC8387172F9E}" interval="1" name="coffee-chats" type="6" refreshedVersion="8" refreshOnLoad="1" saveData="1">
-    <textPr prompt="0" sourceFile="C:\Users\user\Desktop\Github\Job Tracker\coffee-chats.csv" comma="1">
+    <textPr prompt="0" sourceFile="coffee-chats.csv" comma="1">
       <textFields>
         <textField/>
       </textFields>
     </textPr>
   </connection>
   <connection id="3" xr16:uid="{4FF36A1E-BAEF-4FBB-9F60-69CC09100052}" interval="1" name="interview-rounds" type="6" refreshedVersion="8" refreshOnLoad="1" saveData="1">
-    <textPr prompt="0" sourceFile="C:\Users\user\Desktop\Github\Job Tracker\interview-rounds.csv" comma="1">
+    <textPr prompt="0" sourceFile="interview-rounds.csv" comma="1">
       <textFields>
         <textField/>
       </textFields>

</xml_diff>